<commit_message>
5-product test files for WB and Ozon
</commit_message>
<xml_diff>
--- a/test_ozon_export.xlsx
+++ b/test_ozon_export.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,25 +444,15 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Ставка НДС</t>
+          <t>Описание</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Штрихкод</t>
+          <t>Бренд</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
-        <is>
-          <t>Описание</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Бренд</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
         <is>
           <t>Ссылка на главное фото</t>
         </is>
@@ -471,156 +461,210 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>OZ-001</t>
+          <t>POWER-001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>667351366</t>
+          <t>777351366</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Чай Лошадь символ года 2026 черный листовой подарочный Get Joy Китай 50 гр в жестяной шкатулке</t>
+          <t>Power Bank 20000 мАч внешний аккумулятор с быстрой зарядкой USB-C PD Quick Charge 3.0 черный</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>499</t>
+          <t>1899</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>799</t>
+          <t>3499</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>Внешний аккумулятор ёмкостью 20000 мАч. Поддерживает быструю зарядку Quick Charge 3.0 и Power Delivery через USB-C. Два USB-выхода, LED-индикатор заряда. Компактный корпус.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>4601234567800</t>
+          <t>PowerMax</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Подарочный черный чай в жестяной шкатулке. Премиальное качество, насыщенный вкус. Идеальный подарок на Новый год 2026.</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Get Joy</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>https://cdn1.ozone.ru/multimedia/photo1.jpg</t>
+          <t>https://cdn1.ozone.ru/multimedia/powerbank.jpg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>OZ-002</t>
+          <t>TEA-002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>667351367</t>
+          <t>777351367</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Кофе зерновой Бразилия Сантос 1 кг</t>
+          <t>Чай зелёный Jasmine Green крупнолистовой с жасмином 100 пакетиков подарочная упаковка</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1299</t>
+          <t>499</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1999</t>
+          <t>799</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>10%</t>
+          <t>Зелёный чай с натуральным жасмином. 100 пакетиков в индивидуальных конвертах. Подарочная упаковка. Без искусственных ароматизаторов.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>4601234567801</t>
+          <t>GreenLeaf</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>100% арабика. Бразилия Сантос. Средняя обжарка. Идеален для эспрессо и турки.</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>CoffeeTime</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>https://cdn1.ozone.ru/multimedia/photo2.jpg</t>
+          <t>https://cdn1.ozone.ru/multimedia/tea.jpg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>OZ-003</t>
+          <t>COFFEE-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>667351368</t>
+          <t>777351368</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Power Bank 20000 mAh быстрая зарядка USB-C</t>
+          <t>Кофе в зёрнах 100% Арабика Бразилия Сантос свежей обжарки 1 кг</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1899</t>
+          <t>1299</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>1999</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>100% арабика из Бразилии. Средняя обжарка. Свежая обжарка — не более 14 дней до поставки. Плотное тело, шоколадные и ореховые ноты.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>CoffeeTime</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://cdn1.ozone.ru/multimedia/coffee.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>LAMP-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>777351369</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Настольная LED-лампа с сенсорным управлением регулировка яркости и цветовой температуры белая</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2499</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>4499</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Светодиодная настольная лампа с сенсорным управлением. 3 режима яркости и 3 цветовые температуры (тёплый, нейтральный, холодный). Гибкая ножка. USB-питание.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>LightWave</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://cdn1.ozone.ru/multimedia/lamp.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BAG-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>777351370</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Рюкзак городской водонепроницаемый 30 литров отделение для ноутбука 15.6" серый</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>3499</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>4601234567802</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Портативное зарядное устройство 20000 мАч. Поддержка быстрой зарядки QC 3.0 и PD.</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>PowerMax</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>https://cdn1.ozone.ru/multimedia/photo3.jpg</t>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>5999</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Городской рюкзак из водонепроницаемой ткани. Отделение для ноутбука до 15.6 дюймов. Множество карманов, USB-порт для зарядки, спинка с вентиляцией.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>UrbanGear</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://cdn1.ozone.ru/multimedia/backpack.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>